<commit_message>
cleaned up some code, added functionality to create new users
</commit_message>
<xml_diff>
--- a/ParentEmployeeInformation.xlsx
+++ b/ParentEmployeeInformation.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mapheyp\Documents\GitHub\PARS---Standalone-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88F4E2B4-841C-4208-AD5B-DBD0D91E0FAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A766EC74-C524-4170-A850-3048EEC6D132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-180" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="3" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">MAIN!$B$1:$B$366</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">

</xml_diff>